<commit_message>
Update example dataset: add Reach Top 25 (low-chance elite) sheet
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/MIM_TOP25_AND_MORE.xlsx
+++ b/examples/MIM_TOP25_AND_MORE.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 25 Ranked" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Near-Misses (26-40)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy &amp; Deadlines" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read-Me &amp; Flags" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reach Top 25 (LOW-CHANCE)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Near-Misses (26-40)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy &amp; Deadlines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read-Me &amp; Flags" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Top 25 Ranked'!$A$1:$S$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'15 Near-Misses (26-40)'!$A$1:$S$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Reach Top 25 (LOW-CHANCE)'!$A$1:$T$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'15 Near-Misses (26-40)'!$A$1:$S$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +43,10 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
@@ -48,7 +54,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +86,26 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ED7D31"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,8 +153,21 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3007,6 +3046,2652 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:T28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RANK</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PROGRAM</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>COUNTRY</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TIER</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DURATION</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2027 DEADLINE</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ODDS @ GMAT FOCUS 655</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TUITION (2027 EST.)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ALL-IN COST (TUITION+LIVING)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>% INDIAN (EST.)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>STARTING SALARY</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>ROI: RECLAIM ALL COST</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>WORK WHILE STUDYING</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>POST-STUDY VISA</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SPOON-FED /10</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>EAS INDIAN LIVING</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>DATA CONFIDENCE</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>VERDICT (1-LINE)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>STRATEGY FLAG @655</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Quantitative Finance</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>LSE</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>REACH-A</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>10 mo</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Rolling; no hard deadline — apply Nov/Dec 2026; needs-based awards 22 Apr 2027 (CONFIRMED)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>LOW (class skews 700+; hardest LSE finance degree)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>~£53,600 (MSc Finance rate CONFIRMED for 2027/28; QF page 404'd — verify)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>£77-80k</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>~20-25% [est]</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>£55-70k [est] — quant/derivatives: Citi, JPM, UBS, Morgan Stanley + hedge funds (Two Sigma, Optiver)</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>~3.5-4.5 yrs</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk term + unlimited vacation (CONFIRMED)</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>2-yr Graduate Route (CONFIRMED for 2027) + Skilled Worker</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>7/10 — quant firms run dedicated LSE-QF days; small cohort = high offer rates</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>9/10 London</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Tuition CONFIRMED (lse.ac.uk); QF URL + odds EST</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>The anchor reach: strongest quant placement pipeline in the UK</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>RETAKE-TO-700+ (or foreground ML/quant portfolio hard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Mathematical Finance</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>LSE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>REACH-A</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>9-10 mo</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Rolling (verify on LSE course finder)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>LOW-MED (math-heavy; quant aptitude &gt; GMAT; agent-unlisted addition)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>~£53,600 [est — assumed same as MSc Finance, VERIFY]</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>£77-80k</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>~15-25% [est]</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>£55-75k [est] quant/IB</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>~3-4.5 yrs</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR + Skilled Worker</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>7/10</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>9/10 London</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>EST — agent-unlisted addition; verify on course finder</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>LSE's dedicated math-finance degree; retake matters less, math prep matters more</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS + math/quant prep (GMAT not the gate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Financial Economics</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Oxford</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>REACH-A</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>9 mo (early autumn)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>~Jan 2027, 2 rounds [est — site 403'd]</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>LOW (class ~690+ Focus-equiv; most score/pedigree-sensitive of the 7 UK)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>~£60k [est — 2027 unconfirmed]</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>£95-100k</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>~12-18% [est]</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>£60-75k [est] IB/consulting: JPM, Goldman, Citi, Barclays London, MBB</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>~3-4 yrs IF IB onboards</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>6/10 (bank onsites; econ-flavoured, not a placement machine)</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Good (small city; very safe)</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify fees/deadline on ox.ac.uk</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>The name dream reach; economics-adjacent, not a quant desk feed</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>RETAKE-TO-700+ (dream reach; retake strongly advised)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Mathematical Finance</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Oxford</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>REACH-A</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>9 mo</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Rounds ~Jan 2027 [verify]</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>LOWEST on this list (tiny ~30-40 cohort; quant gate; grades + math)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>~£60-65k [est — VERIFY]</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>£95-100k</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>not published, ~10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>£60-80k [est] quant/IB</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>~3-4 yrs</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>6/10</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Good (Oxford)</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>EST — agent-unlisted addition; verify program page</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>Oxford's hardest finance degree; math ability is the gate, not GMAT</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS + strong quant portfolio (P1-P6) — retake won't fix the gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Cambridge</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>REACH-A</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>12 mo</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>~early Jan 2027 [est — verify cam.ac.uk]</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>LOW (class ~680-720 trad / ~660-700+ Focus; 655 at/below median)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>~£55-58k [est — 2027 unconfirmed]</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>£88-92k</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>~10-15% [est] (US/intl-heavy cohort)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>£45-55k [est] — GS/JPM/Citi/Barclays associates, MBB, Big 4</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>~4-5.5 yrs</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (CamFinance bank hiring days)</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>G5 name with a thinner pipeline than LSE; you buy prestige, not placement density</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>RETAKE-TO-700+ (recommended)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Quantitative Finance</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>UZH (Zurich)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>~15 Feb 2027 [est — verify uzh.ch]</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>LOW (NO GMAT — transcript gate: math/quant fit; ~20-30% admit [est])</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>CHF ~1,400 TOTAL tuition (public) [est]</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>CHF 25-28k (living dominates)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>5-8% [est] (cohort ~40/yr)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>CHF 95-120k [est] — UBS/JB/Pictet quant analysts (highest DACH salary)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>~1-1.5 yrs post-grad — CONDITIONAL on B-permit (0 work hrs while studying, NO job-search visa)</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>0 HOURS (CH, 3rd-country)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>NONE — B permit, employer-tied, canton salary thresholds</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>4/10 (self-market; UBS campus days are invite-only)</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Cold, very expensive, small Indian community (~8-10k Zurich)</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>EST — fees page 404'd; verify</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>ROI king of the whole list if you get in; strictest immigration catch</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (grades-gated — retake useless); pre-line the job offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance &amp; Banking</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>HEC Paris</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs (M1 entry)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>4-5 rounds; early ~mid-Dec 2026 [est — HEC MIM R2 26 Nov is a different program]</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>MED-LOW (class ~680-710 [est]; 2y Amazon top-5% + founder P&amp;L compensate)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>~€33.5-36k/yr [est — HEC publishes no per-program fee; ~€70-75k for 2 yrs]</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>~€105-115k all-in</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est]</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>€60-75k [est] — BNP, SocGen, Amundi, PwC/KPMG, JPM Paris, LVMH treasury</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>~1.7-2 yrs incl. part-time work (964h/yr)</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>964 h/yr (~48 h/wk legal)</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>APS 12-mo → Passeport Talent</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>8/10 (bank on-site days in week 1 of term; ~85-90% placed in 4-6 mo [est])</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Good (Paris 8/10)</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Fees EST (not published per program); ~7% uni-wide acceptance [est]</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>Most elite FR brand; 655 is 30-45 pts below class median — real risk</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (borderline; +20-30 pts would move it to MED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Quantitative Finance</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ESSEC</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs (M1 entry)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>R1 ~late Jan 2027; final ~Mar-Apr [est]</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>MED-LOW (class ~660-690 [est]; 655 at/below median; quant creds help)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>~€33-36k/yr [est] → ~€70k 2-yr</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>~€95-100k (Cergy living much cheaper than Paris)</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est]</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>€55-70k [est] — PwC/EY Paris, BNP, LVMH, Danone, Crédit Agricole, JPM Paris</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>~1.7 yrs</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>964 h/yr</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>APS 12-mo</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (strong office; AMCs less centralized than HEC; many land jobs via networks)</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Fair (Cergy dorm town; 30-40 min to Paris)</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify essec.edu</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>Genuinely CFA/FRM + Python/C++ quant curriculum; cheaper base than HEC; ESSEC Global Excellence up to ~40% tuition [est]</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Quantitative Finance</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Bocconi (SDA)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>R1 ~mid-Mar 2027; R2 ~late Jun [est]</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>MED-LOW (APTITUDE TEST-gated, not GMAT; hardest Bocconi track; 8.5/10 workable)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>~€16.5-18k/yr [est → ~€33-36k 2-yr] — CONFLICTS with earlier agent's €44-47k/yr; VERIFY on unibocconi.it</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>~€58-65k all-in</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est] (large Indian presence in finance tracks)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>€45-60k [est] — Intesa Sanpaolo, UniCredit, BNP Italy, JPM Milan (+ GS/BlackRock/KKR Italy)</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>~14-20 mo post-grad (net ~€40-48k after 20h/wk offsets)</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>12-mo 'permesso per ricerca lavoro' [verify]</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>8/10 (quant/finance on-sites; structured internships)</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>BEST in Europe (Milan ~25-30k Indians; veg everywhere; 25-30k community)</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>EST — fee conflict flagged; verify both structure + fees</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>Best EU quant brand + best scholarship odds (Excellence up to 100% tuition) + best Indian living</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS — prep the aptitude test, not a GMAT retake</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>NUS</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>12 mo</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Single rolling round ~Sep-Oct 2026 → Feb 2027 [est — confirm intake month]</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>MED (GMAT NOT a gate; GPA + experience driven; 655 irrelevant)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>~S$145-150k [est — 2025 was S$131,750 incl GST; fees page empty, verify]</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>S$165-175k (~INR 10.6-11.2M)</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>~20-30% [est]</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>S$50-55k/yr [est] — DBS, OCBC, GIC, Citi/JPM SG (+ UOB, Big 4)</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>~3.2 yrs — weakest SG ROI (no PWP if 12-mo claim holds)</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>NONE if agent's PWP-18-month claim holds [UNRESOLVED — NUS FAQ confirms 16h/wk for intl postgrad generally; confirm at MOM]</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>EP + COMPASS (NUS bonus institution) + 6-mo SG Work Pass (Feb 2025, NUS on recognised list)</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (career services + on-campus SG bank/Big-4; small market)</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Tuition EST (page empty); PWP claim unverified</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>Most prestigious APAC brand but priciest SG quant + work-rights question mark</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (GMAT not gate) — weight the cost before filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>HKUST</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>REACH-B</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>12 mo (Sep)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>P1 11 OCT 2026, P2 29 Nov 2026, P3 10 Jan 2027, P4 28 Feb 2027 — CONFIRMED (mfin.hkust.edu.hk)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>LOW (no published cutoff; elite quant pool, 655 at/below median; Amazon risk + AWS certs differentiate)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>~HK$180-190k [est — recent ~HK$169k; verify]</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>HK$335-345k (~INR 2.8-2.9M)</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>~15-25% [est]</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>HK$400-500k [est] — JPM HK, Goldman HK, BofA, SSG (+ Citi/HSBC/UBS HK)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>~1-1.5 yrs — best tuition-recovery math in APAC reach</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>NO HOUR CAP; full-time from ~month 7 (HK rules)</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>IANG 2 yrs (renewable 3+2)</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>8/10 — US banks run on-campus recruiting + return-offer conversion; strongest classic APAC launchpad</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (hot-humid, very safe; Indian food in Kowloon/Central)</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Deadlines CONFIRMED; fees/salaries EST</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>Only reach APAC where reclaim-while-studying is real; entrance scholarship HK$50-100k [est]</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS in P1 (11 Oct 2026) — retake is marginal, class-median is the gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Fintech</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>HKUST</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>12 mo (Sep)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Same 4 phases as MSc Finance [per-program dates est]</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>MED — HIGHEST chance of the 5 APAC (GMAT not gate; AWS ML/DE + Amazon risk + tech founder = exact fit)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>~HK$150-170k [est]</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>HK$300k (~INR 2.5M) — cheapest total of the 5</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>~20-25% [est]</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>HK$350-450k [est] — HSBC Fintech, JPM, DBS Fintech SG, Ant International</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>~1-1.5 yrs</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>full-time from ~month 7</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>IANG 2 yrs</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>8/10 (same HKUST machine; dual SG/HK placements)</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>7/10</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>EST (deadlines structure same as MScF)</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>Tech-adjacent finance at the cheapest total; title less pure-finance for bank desks</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (best-fit reach program on this list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance / MSc in Asset Management</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Cass Business School (City, U. London)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>12 mo</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>~Jan-Feb 2027 [est — verify]</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>MED-HIGH (score-tolerant; employer-pipeline-driven; 655 fine with work ex)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>~£35-40k [est — verify]</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>£58-64k — cheapest of the 7 UK</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>~25-35% [est] — highest South Asian share of the 7</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>£45-55k [est] — JPM, Citi, BofA, Big 4 + City/prop desks</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>~2.5-3.5 yrs — best raw ROI of the 7</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>9/10 — MOST SPOON-FED of the UK 7; banks hire by quota; highest IB offer-per-head ratio</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Good (London)</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify fees; placement [est]</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>Brand weakest of the UK 7, but the strongest placement engine — in the City the name matters more than in India</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (safest elite-UK pick)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>UCL</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>12 mo</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>~late Jan 2027 [est — multi-round]</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>MED-HIGH (most score-permissive elite option; 655 + Amazon + founder = solid)</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>~£40-45k [est — verify]</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>£63-68k</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>~20-25% [est] — largest South Asian cohort of the 7</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>£45-55k [est] — Citi, HSBC, JPM, Big 4, KPMG EBG</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>~3-4 yrs — cheapest top-5 path</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>8/10 (career fair well-attended by banks; you hustle for the same onsites)</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Good (London)</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>'LSE-lite': less alumni density at IB desks; biggest risk is the program name, not the pipeline</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Imperial College London</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>12 mo</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>~Jan 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>MED (wider band; actively recruits career-changers with work ex — Amazon 2y + top-5% + promotion hits profile)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>~£44-48k [est — verify]</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>£70-74k</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est]</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>£50-60k [est] — JPM, Citi, BofA London, MBB, Big 4</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>~3-4 yrs — best cost-adjusted London option</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk + vacation</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2-yr GR</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (bank onsites solid but thinner than LSE)</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>9/10 London</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>Value pick over LSE for career-changers; G5 name + strong CV culture</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (most realistic G5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Quantitative Finance</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>NTU Nanyang</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>12 mo (Sep)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>~2 rounds; R1 ~Nov 2026-Jan 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>MED (not GMAT-gated; NTU's own quant label — verify program exists for 2027)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>~S$95-105k [est — VERIFY]</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>S$115-125k (~INR 7.4-8M)</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>~10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>S$48-58k [est] — OCBC/UOB quant, MAS, Big 4</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>~2.4-2.6 yrs</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>NONE if PWP-18m claim holds [UNRESOLVED]</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>EP + COMPASS + 6-mo SG Work Pass</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>6.5/10</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>EST — agent-flagged program; verify on ntu.edu.sg</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>If 'quant' branding matters more than NUS brand, this beats NUS MScF on fit at a similar cost</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>NTU Nanyang</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>12 mo (Sep)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>R1 ~Nov 2026-Jan 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>MED (highest of the 2 SG MScF schools; less GPA-elite pool than NUS)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>~S$100-105k [est]</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>S$120-128k (~INR 7.7-8.2M)</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>~10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>S$45-50k [est] — OCBC, UOB, Straits Capital, Big 4, MAS</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>~2.6 yrs</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>NONE if PWP claim holds [UNRESOLVED]</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>EP + COMPASS</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>6/10 (smaller bank presence than NUS)</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>The cheaper SG sibling; SOM merit award S$5-10k [est]</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance (quant track)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>TUM School of Management</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs (120 ECTS, full-English)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Winter window Sep 2026 - 15 Jan 2027 [est — confirm]</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>MED (NO GMAT — CGPA gate: 8.5/10 ≈ 2.5-2.6 German grade, at/just below ~2.5-3.0 cutoff [est])</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>~€12,000 TOTAL tuition (public; ~€500/sem admin) [est]</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>~€36-40k (living dominates, 2 yrs)</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est] (class ~40-60/yr; TUM ~25-30% Indian overall)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>€55-65k [est] — Allianz HQ, DB DACH, PwC/EY/KPMG Munich, ING, BMW corp-fin</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1 yr post-grad — best absolute ROI in DE</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>140 full days/yr (~280 h)</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>18-mo job-search + Blue Card</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>6/10 (bank on-campuses less frequent than HEC; DACH career fairs in FR/MU)</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Good (Munich: ~30k Indians; housing crisis — wait 2-4 mo for a flat)</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify program page + fees</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>Public + rigorous + DACH bank pipeline; 'IIT of Germany'; GMAT irrelevant</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (grades-gated — retake useless)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurt School</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>1 yr (Sep)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Rolling ~15 Jul 2027; interview rounds earlier [est]</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>MED (NO GMAT — interview + motivation + experience; 2y Amazon = strong signal)</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>~€14-16k [est — one of cheapest private DE]</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>~€28-30k</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>~8-12% [est]</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>€52-60k [est] — Deutsche Bank + Commerzbank HQ town, ING Frankfurt, KPMG/PwC Frankfurt, UniCredit</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1 yr — excellent ROI, lowest DE-private cost</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>140 days/yr</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>18-mo job-search + blue-card track</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (Career Center books DE-bank on-site days; IB/CorpFin intern conversions)</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>Good (compact, safe, ~50 veg spots, ~15k Indians in region)</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify fees page</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>ECB/BaFin city; junior hiring soft at DB/Commerzbank 2024-26 but quant/IB roles resilient; merit 25-50% for top ~10% [est]</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>WHU</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>REACH-C</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1 yr (Sep)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Rolling; final ~15 Apr 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>MED (NO GMAT — internal evaluation + interviews; Amazon 2y ideal)</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>~€30-33k [est]</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>~€42-45k (Koblenz living)</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>~10-12% [est]</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>€55-65k [est] — Deutsche Bank, PwC Frankfurt, KPMG, ING, Allianz, UBS Munich</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1 yr post-grad</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>140 days/yr</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>18-mo job-search</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>7/10 (WHU Finance Society gets real bank off-sites)</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>Fair (small town; 20 min to Frankfurt's Indian food; ~5k Indians in RLP)</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Strong DE-IB niche; location + small cohort = ceiling; Global Excellence up to 50% (~5% of class) [est]</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (target the 75% Responsible Leader if offered for MSc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>EDHEC</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>REACH-D</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>1 yr</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>3 rounds; final ~late Feb 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>MED — HIGHEST chance of the FR BGA trio (class ~630-660 [est]; 655 AT/ABOVE median)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>~€19.5-22k [est] (MiM fee EUR 51,250 is a different program — CONFIRMED)</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>~€32-36k (cheap Lille living)</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>~10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>€48-58k [est] — PwC/KPMG, SocGen Lille, Danone, Capgemini, Natixis</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>&lt;1 yr — best pure ROI of the FR BGA</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>964 h/yr</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>APS 12-mo</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>6/10 (smaller career office; more self-marketing than HEC)</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Good (Lille: compact, safe, cheap)</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>MiM fee CONFIRMED; MScF fee EST</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Value Grande École; your 655 clears it comfortably</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (highest chance in France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Finance (Quantitative track)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>EPFL (Lausanne)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>REACH-D</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>1 yr</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Round 1 ~15 Jan 2027 (priority); round 2 end-March [est]</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>LOW-MED (NO GMAT; engineers welcomed — CSE + risk-quant on-track; 8.5 borderline-competitive)</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>CHF 3,500-4,000/yr (non-Swiss) [est]</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>CHF 26-32k total</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>CHF 85-105k [est] — Pictet, Lombard Odier, UBS (Geneva), BNP Paribas WM, Swiss Re</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>~10-12 mo post-grad IF B permit pre-arrived (0 work hrs + no search visa)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>0 HOURS (CH)</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>NONE (B permit, Vaud/Geneva cantons)</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>5/10 (career fairs + on-campus; still largely self-marketing)</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>Fair (4-6k Indians; French in daily life; Geneva 20 min by train)</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify track naming + fees</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>Credible cheaper ETH-alternative; Geneva wealth houses hire EPFL quant grads; Excellence Scholarship 25-100% tuition (low probability at 8.5/10)</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (grades-gated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Banking &amp; Finance (dual degree)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Bocconi (SDA)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>REACH-D</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>R1 ~mid-Mar 2027 [verify]</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>MED (test-gated; dual degree with a partner school adds a 2nd credential)</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>~€18k/yr [est — same fee conflict as row 9, VERIFY]</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>~€55-60k all-in</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>~15-20% [est]</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>€45-60k [est] — IB/PE analyst: UniCredit, Intesa, UBS/JPM Milan, KKR Italy</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>~1.5-2 yrs</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>12-mo search permit</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>8/10 (strong career service + on-campus quant/finance on-sites)</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>BEST in Europe (Milan: ~25-30k Indians; veg everywhere)</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>EST — agent-unlisted addition; verify structure on unibocconi.it</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>The IB-flavoured Bocconi degree with dual-credential leverage; best scholarship odds in Italy</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (test prep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Financial &amp; Insurance Mathematics</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>KTH (Stockholm)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>REACH-D</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>1 yr (60 ECTS)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>~15 Jan 2027 non-EU portal [est]</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>MED-LOW (NO GMAT — specific math-credit gate: calculus/linear algebra/probability ~45-60 cr [est]; few non-EU slots)</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>SEK 157-240k (~€14-21k) [est — verify 2027 rate]</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>SEK 350-400k (~€30-35k)</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>15-25% [est] (big Stockholm Indian community)</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>SEK 350-450k [est] insurance/actuarial; 450-550k [est] at SEB/Nordea quant desks</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>~10-14 mo post-grad — cheapest Nordic ROI</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>12-mo job-search (Sweden = EU)</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>4/10 (insurers know KTH; self-market to SEB/Nordea/APG/Alecta/Skandia)</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>Fair-to-good (8-10k Indians; dark winter; Systembolaget alcohol rules)</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>EST — verify credit reqs + fees</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>Hard-quant degree; domestic insurance/asset-mgmt pipeline (APG, Alecta, Skandia); SISG scholarship = best funding shot</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (credit-gated — check your course list for the math credits first)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>MSc in Economics (Finance specialisation)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Aalto (Helsinki)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>REACH-D</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2 yrs</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Main round ~15 Apr 2027 [est]</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>MED — HIGHEST chance of the 6 CH/IT/Nordic (grades-based; 8.5 CSE fits comfortably)</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>~€16k/yr [est] → €32-34k 2-yr</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>~€58-62k (Helsinki)</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>10-15% [est]</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>€36-45k [est] — OP Financial, Nordea, SEB, S-Pankki (+ EY/PwC/Danske)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>~16-20 mo post-grad (lowest salaries in the set)</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>20h/wk</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>6-mo job-search [verify — some sources say up to 12]</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>4/10 (small employer base; many grads pivot to data/tech)</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Fair (4-6k Indians; veg limited; very dark Dec; small polite society)</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>EST</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>Good value + Aalto International Talent Scholarship (auto-awarded 25-100% — best size/odds combo in Nordics); Finnish finance market too small for quant depth</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>APPLY-AS-IS (highest chance + best Nordic scholarship odds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>TIER LEGEND: REACH-A = dream/LOW (1-2 in 10 admitted at 655 or grade-gated)  |  REACH-B = elite quant, MED-LOW  |  REACH-C = elite &amp; attainable, MED+  |  REACH-D = value quant, MED+  —  All 25 strictly above the original Top 25 in prestige. STRATEGY FLAG column: RETAKE-TO-700+ = GMAT retake materially improves odds; APPLY-AS-IS = grades/test/other gate, retake won't fix it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:T26"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4551,7 +7236,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4565,456 +7250,456 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>SECTION</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>DETAIL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>APPLICATION WAVES (Dec 2026 - Mar 2027)</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr"/>
+      <c r="B2" s="14" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Wave 1 (Nov-Dec 2026):</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>HEC R2 (26 Nov 2026 - CONFIRMED), IE R1 (15 Nov 2026 - CONFIRMED), ESSEC rolling, WHU scholarship round (31 Jan — apply early)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Wave 2 (Jan 2027):</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Imperial (6 Jan - CONFIRMED), NTU Jan round (~31 Jan), LSE single round (~mid-Jan), Cambridge (~early Jan), WHU general (~31 Jan)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Wave 3 (Feb-Mar 2027):</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>SMU (~Mar 31), HKUST (~Mar 15), HKU (~Mar 31), Bocconi (~late Feb-Mar), Erasmus/Tilburg (~Feb-Mar), Maastricht (~Jun - non-EU window)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Wave 4 (Apr-Jul 2027):</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Ca' Foscari single call, CEU, DCU rolling, TUM (~Jul), WU/UZH/ETH/St. Gallen (~Mar-May)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>ANCHOR SET (Tier 1 = 5 + 1)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr"/>
+      <c r="B7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Apply first:</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>NUS, DCU, HKUST, SMU, TUM + IE Madrid (EU all-rounder)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Reach layer:</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>HKU MScF, LSE, HEC, Cambridge</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Safety layer:</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>NTU, Warwick, DCU, WU, Aalto, Erasmus, Tilburg, Ca' Foscari</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>SCHOLARSHIP LEVERAGE (apply early!)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr"/>
+      <c r="B11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>WHU Responsible Leader 75% (31 Jan deadline, CONFIRMED)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Single highest-leverage application on the whole list — cuts EUR 75k to ~EUR 20-25k</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>KTH 1-2 yr tuition coverage</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Verified tiered scholarship from KTH admissions page</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>IE R1 merit (EUR 15-35k est.)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Early round = best odds</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>NUS/NTU/SMU merit awards</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>S$10-30k band; no India-specific MIM scholarships in SG</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>ESSEC apprenticeship track</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Employer PAYS tuition + salary while studying — verify which track it covers before 2027</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>RECLAIM-MONEY-WHILE-STUDYING LADDER</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr"/>
+      <c r="B17" s="14" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>1st: HK (full-time from month 7)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>~INR 10-15L back in final semester alone</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>2nd: Ireland (full-time all year)</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Best for staying in EU</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>3rd: France (964 h/yr ≈ 48h/wk)</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Best PT regime in continental EU</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>4th</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Spain (30h/wk) / SG PWP (16-24h/wk) / UK+NL+Nordics (16-20h/wk) / Germany (140 days/yr)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>0th: Switzerland &amp; UAE (0 hours)</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Cannot work at all during study</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>POST-STUDY JOB-SEARCH LADDER (longest first)</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr"/>
+      <c r="B23" s="14" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Ireland 24-mo</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Stamp 1G, verified</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>UK 24-mo</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Graduate Route</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>Germany 18-mo</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Aufenthaltstitel zur Jobsuche</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>France 12-mo</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>APS -&gt; then Passeport Talent</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Netherlands 12-mo</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>zoekjaar, RENEWABLE, apply within 3 yrs</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Spain / Sweden / Denmark 12-mo</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Denmark adds 1-yr extension</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Austria / Finland 6-mo</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Shortest</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Switzerland / UAE: none</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>Must already hold an offer</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>BEFORE YOU PAY ANY FEE (re-verify list)</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr"/>
+      <c r="B32" s="14" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>NYU Abu Dhabi: does a finance MSc even exist + post-2028 delivery model (nyuad.edu)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>St. Gallen SFA: 1-yr fee — CHF 42-45k vs CHF 90-100k conflict (sfa-egi.ch)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>ESSEC: 1-yr MiF tuition vs 2-yr Intensive track (essec.edu)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>Bocconi: 2027 fee + entrance exam requirement at 655 Focus (sdabocconi.it)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>Spain 30h/wk work rule with your consulate (2023 consolidated text)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>Sweden 12 vs 18-month job-search permit (Migrationsverket)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>UK 2027 Skilled Worker salary threshold + Graduate Route still 2 yrs</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>SG EP/COMPASS 2027 salary floor (mom.gov.sg) and HK IANG rules (immd.gov.hk)</t>
         </is>
@@ -5025,7 +7710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5039,152 +7724,152 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>TOPIC</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>CANDIDATE</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Vedant Konde — Indian, 21, B.E. Comp Eng 8.5/10, GMAT FOCUS 655, 2 yrs Amazon Risk Specialist (top-5% SME), chess-venture founder, AWS ML+DE certs. Sep 2027 intake. India/US/Australia excluded.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>FX CONVERSIONS USED</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>1 SGD ~ INR 6.4; 1 HKD ~ INR 0.84; 1 EUR ~ INR 98; 1 CHF ~ INR 88; 1 GBP ~ INR 160; 1 SEK ~ EUR 0.09. Update before financial planning.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>CONFIDENCE LEGEND</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr"/>
+      <c r="B4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>CONFIRMED</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Verified against official program/university pages this research cycle (URLs in MIM_TOP25_REPORT.md). Safe to plan around.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>EST / [unverified]</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>2024-25 vintage or agent estimate; search backend was throttled. Re-check on the official 2027 intake page BEFORE paying any application fee.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>[2024-25]</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Explicitly last-year published figures carried over; expect +5-8% for 2027.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>VERIFY</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Fact could not be confirmed by any source this cycle (e.g., NYUAD finance MSc existence, St. Gallen 1-yr fee).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>SOURCES</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Confirmed-live: NUS MiM fees (mim.nus.edu.sg), Imperial (imperial.ac.uk), WHU scholarship+avg salary (whu.edu), HEC fees/rounds/salary (hec.edu, FT 2026), ESSEC 2-yr (3rd-party), IE everything (ie.edu), Maastricht fee (maastrichtuniversity.nl), CBS fee (cbs.dk), EDHEC fee (edhec.edu), KTH fee+scholarships (kth.se), SSE fee+GMAT floor (hhs.se), Ireland Stamp 1G (irishimmigration.ie + TCD), Germany 18-mo (Berliner Welcome Center), Sweden 12-mo (Migrationsverket), NL 3-yr renewal (UvA/IND).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>KNOWN CONFLICTS</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>St. Gallen 1-yr fee: CHF 42-45k vs CHF 90-100k (different programs) — verify. Sweden job-search: 12 vs 18 months — verify.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>OPEN ITEMS</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>NYUAD finance MSc existence; ESSEC 1-yr vs 2-yr track cost; Spain 30h/wk consulate confirmation; UK 2027 Skilled Worker threshold; SG 2027 EP salary floor.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>DISCLAIMER</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>All marked EST figures are 2024-25 data or agent estimates; the search backend was throttled for several regions. This sheet informs decisions but is not a guarantee — verify each figure on the official 2027 intake page before paying fees.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>COMPANION DOC</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>MIM_TOP25_REPORT.md (full 13-dimension narrative per program + source URLs). STRATEGY_2027_APPLY.md (project plan + portfolio P1-P6).</t>
         </is>

</xml_diff>